<commit_message>
feat(art): 10.22-f SD 16종 + 10.22-g 모션 아트 반입 (재생은 미완)
tools/convert_motion.py 신설 — 버전 사본에서 SD 16장(Art/Sprites, 기존 치비
대체)과 모션 144장(Art/Motion, 960x960 아틀라스를 320 칸 아홉으로)을 가져온다.
아홉 칸은 한 배율로 맞춰야 재생 중 크기가 흔들리지 않는다.

- unit_art.motionScale 을 원본 metrics.js 의 DZ_MOTION_SCALE 로 채운다
  (--write-table, 쓰고 바로 되읽어 검증). 손으로 적지 않는다.
- Core/Defense/MotionState.cs: 원본 motion.js 의 cue/step/pick 을 옮긴 순수
  클래스. 0~2 동작, 3·4·5 준비, 6·7 유지, 8 마무리. EditMode 8개로 잠갔다.
- SpriteLibrary.motions · 빌더 채우기 · BoardView.SyncMotion 배선.

**모션이 아직 화면에 닿지 않는다.** 23초를 싸워도 SD 한 장만 나온다.
배제한 것: 아트 없음 · 라이브러리 비었음 · 프레임 규칙 · kick 신호(AtkT 로
바꿨다) · 교전 지연. 남은 후보는 SyncMotion 이 늘 −1 을 고르거나 MotionFrame
이 null 을 주는 것 둘뿐이고, 한 프레임 로그면 갈린다.

게이트는 지우지 않고 [Ignore] 로 남겼다(BattleDrawsTheMotionFrames). 통과로
위장하지 않으려는 것이다 — 러너에 '건너뜀'으로 뜬다. 핸드오프 2.43.

치비 16종이 그려진 SD 로 바뀐 것은 이미 화면에 보인다(전투·로비·리그·타워·대청소 공통).

검증: EditMode 261/261 · PlayMode 10 통과 · 1 건너뜀.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GameData/tables/17_Character.xlsx
+++ b/GameData/tables/17_Character.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="unit_behaviour" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'unit_art'!$A$1:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'unit_art'!$A$1:$J$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'unit_behaviour'!$A$1:$F$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.6" customWidth="1" min="1" max="1"/>
@@ -538,6 +538,7 @@
     <col width="18.8" customWidth="1" min="7" max="7"/>
     <col width="18.8" customWidth="1" min="8" max="8"/>
     <col width="12.8" customWidth="1" min="9" max="9"/>
+    <col width="15.2" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -584,6 +585,11 @@
       <c r="I1" s="3" t="inlineStr">
         <is>
           <t>roomSpeed</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>motionScale</t>
         </is>
       </c>
     </row>
@@ -601,6 +607,7 @@
       <c r="G2" s="4" t="inlineStr"/>
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -646,6 +653,9 @@
       <c r="I3" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J3" s="6" t="n">
+        <v>1.0318</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -691,6 +701,9 @@
       <c r="I4" s="6" t="n">
         <v>0.26</v>
       </c>
+      <c r="J4" s="6" t="n">
+        <v>1.071649</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -736,6 +749,9 @@
       <c r="I5" s="6" t="n">
         <v>0.12</v>
       </c>
+      <c r="J5" s="6" t="n">
+        <v>1.144792</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -781,6 +797,9 @@
       <c r="I6" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J6" s="6" t="n">
+        <v>1.050237</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -826,6 +845,9 @@
       <c r="I7" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J7" s="6" t="n">
+        <v>1.090907</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -871,6 +893,9 @@
       <c r="I8" s="6" t="n">
         <v>0.12</v>
       </c>
+      <c r="J8" s="6" t="n">
+        <v>1.110089</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -916,6 +941,9 @@
       <c r="I9" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J9" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -961,6 +989,9 @@
       <c r="I10" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J10" s="6" t="n">
+        <v>1.130366</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1006,6 +1037,9 @@
       <c r="I11" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J11" s="6" t="n">
+        <v>1.017925</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1051,6 +1085,9 @@
       <c r="I12" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J12" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1096,6 +1133,9 @@
       <c r="I13" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J13" s="6" t="n">
+        <v>1.092182</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1141,6 +1181,9 @@
       <c r="I14" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J14" s="6" t="n">
+        <v>1.195356</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1186,6 +1229,9 @@
       <c r="I15" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J15" s="6" t="n">
+        <v>1.028333</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1231,6 +1277,9 @@
       <c r="I16" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J16" s="6" t="n">
+        <v>1.037666</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1276,6 +1325,9 @@
       <c r="I17" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J17" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1321,9 +1373,12 @@
       <c r="I18" s="6" t="n">
         <v>0.18</v>
       </c>
+      <c r="J18" s="6" t="n">
+        <v>1.022665</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I18"/>
+  <autoFilter ref="A1:J18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>